<commit_message>
Programming lever resolved: +$500/wk assumed, baked into revenue base
Slide 6 programming card: placeholder '$xxK -> $xxK' replaced with
'+$500/wk' and a no-double-count note. Tie-out flag cleared (was the
last unmodeled claim); Bridge lever memo updated. No numeric model
changes - the traffic support is already inside the Act/For-based
revenue.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VCQW3YoSqaJfwSKLPDyQy8
</commit_message>
<xml_diff>
--- a/Method_Operating_Model_2027_21.xlsx
+++ b/Method_Operating_Model_2027_21.xlsx
@@ -48,7 +48,7 @@
     <numFmt numFmtId="170" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="171" formatCode="\$#,##0;;\–"/>
   </numFmts>
-  <fonts count="44">
+  <fonts count="45">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -374,6 +374,10 @@
       <color rgb="FF2F5496"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -470,7 +474,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="350">
+  <cellXfs count="351">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1519,6 +1523,9 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1773,7 +1780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="177" min="1" max="1"/>
@@ -2304,17 +2311,17 @@
       </c>
       <c r="C20" s="183" t="inlineStr">
         <is>
-          <t>$xxK → $xxK</t>
+          <t>+$500/wk</t>
         </is>
       </c>
       <c r="D20" s="180" t="inlineStr">
         <is>
-          <t>NOT MODELED</t>
-        </is>
-      </c>
-      <c r="F20" s="186" t="inlineStr">
-        <is>
-          <t>⚠ still placeholder in deck AND absent from model — needs event cost/revenue data</t>
+          <t>assumption — baked into the revenue base</t>
+        </is>
+      </c>
+      <c r="F20" s="350" t="inlineStr">
+        <is>
+          <t>✓ by convention: 2x/month activations assumed to sustain ~$500/wk of traffic already counted in the Act/For-based revenue; no separate lever, no double-count</t>
         </is>
       </c>
     </row>
@@ -2810,11 +2817,9 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="178">
       <c r="A38" s="180" t="n"/>
     </row>
-    <row r="39"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -36534,7 +36539,11 @@
       <c r="H14" s="196" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="178">
-      <c r="A15" s="196" t="n"/>
+      <c r="A15" s="350" t="inlineStr">
+        <is>
+          <t>LW — Programming: 2x/month activations assumed to sustain ~$500/wk of traffic ALREADY included in the revenue base (no incremental revenue modeled)</t>
+        </is>
+      </c>
       <c r="B15" s="196" t="n"/>
       <c r="C15" s="196" t="n"/>
       <c r="D15" s="196" t="n"/>

</xml_diff>